<commit_message>
Cap nhat live-show (badge xanh, dem nguoc khai mac), Excel to cam o nhap tay, va tom tat du an
</commit_message>
<xml_diff>
--- a/Quan_ly_hoi_thao_Final.xlsx
+++ b/Quan_ly_hoi_thao_Final.xlsx
@@ -30,7 +30,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="hh:mm"/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="25">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -190,8 +190,14 @@
       <color rgb="FF000000"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF000000"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -245,6 +251,11 @@
         <fgColor rgb="FF1F3864"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFA500"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -288,7 +299,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -370,6 +381,15 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="24" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -561,7 +581,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="en-US"/>
               </a:p>
@@ -745,7 +765,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -836,7 +856,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -869,7 +889,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
@@ -1234,7 +1254,7 @@
       <c r="A8" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="41" t="inlineStr">
         <is>
           <t>10:15</t>
         </is>
@@ -3935,7 +3955,7 @@
           <t>Tên thành viên</t>
         </is>
       </c>
-      <c r="D6" s="1" t="inlineStr">
+      <c r="D6" s="42" t="inlineStr">
         <is>
           <t>Thứ tự bị loại
 (để trống nếu vô địch)</t>
@@ -3951,7 +3971,7 @@
           <t>Điểm</t>
         </is>
       </c>
-      <c r="G6" s="1" t="inlineStr">
+      <c r="G6" s="42" t="inlineStr">
         <is>
           <t>Ghi chú (thẻ đã dùng)</t>
         </is>
@@ -6945,19 +6965,19 @@
           <t>Đội 2</t>
         </is>
       </c>
-      <c r="F4" s="1" t="inlineStr">
+      <c r="F4" s="42" t="inlineStr">
         <is>
           <t>Chỉ số
 Đội 1</t>
         </is>
       </c>
-      <c r="G4" s="1" t="inlineStr">
+      <c r="G4" s="42" t="inlineStr">
         <is>
           <t>Chỉ số
 Đội 2</t>
         </is>
       </c>
-      <c r="H4" s="1" t="inlineStr">
+      <c r="H4" s="42" t="inlineStr">
         <is>
           <t>Thắng trực tiếp
 (Nữ hoàng bị hạ / phạm luật)</t>
@@ -6973,7 +6993,7 @@
           <t>Đội thua</t>
         </is>
       </c>
-      <c r="K4" s="1" t="inlineStr">
+      <c r="K4" s="42" t="inlineStr">
         <is>
           <t>Ghi chú</t>
         </is>
@@ -6983,7 +7003,7 @@
           <t>Đang thi đấu?</t>
         </is>
       </c>
-      <c r="M4" s="27" t="inlineStr">
+      <c r="M4" s="43" t="inlineStr">
         <is>
           <t>Đang thi đấu (nhập tay)</t>
         </is>
@@ -12059,7 +12079,7 @@
           <t>Đội 2</t>
         </is>
       </c>
-      <c r="E4" s="1" t="inlineStr">
+      <c r="E4" s="42" t="inlineStr">
         <is>
           <t>Đội thắng</t>
         </is>
@@ -12084,22 +12104,22 @@
           <t>Đang thi đấu?</t>
         </is>
       </c>
-      <c r="J4" s="27" t="inlineStr">
+      <c r="J4" s="43" t="inlineStr">
         <is>
           <t>Tên TV vòng sau 1</t>
         </is>
       </c>
-      <c r="K4" s="27" t="inlineStr">
+      <c r="K4" s="43" t="inlineStr">
         <is>
           <t>Tên TV vòng sau 2</t>
         </is>
       </c>
-      <c r="L4" s="27" t="inlineStr">
+      <c r="L4" s="43" t="inlineStr">
         <is>
           <t>Tên TV vòng sau 3</t>
         </is>
       </c>
-      <c r="M4" s="27" t="inlineStr">
+      <c r="M4" s="43" t="inlineStr">
         <is>
           <t>Đang thi đấu (nhập tay)</t>
         </is>
@@ -15398,15 +15418,15 @@
     <mergeCell ref="A49:F49"/>
     <mergeCell ref="A94:F94"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A124:F124"/>
     <mergeCell ref="A79:F79"/>
+    <mergeCell ref="A64:F64"/>
     <mergeCell ref="A34:F34"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A139:F139"/>
     <mergeCell ref="A154:F154"/>
     <mergeCell ref="A19:G19"/>
     <mergeCell ref="A109:F109"/>
-    <mergeCell ref="A64:F64"/>
+    <mergeCell ref="A124:F124"/>
     <mergeCell ref="A17:H17"/>
   </mergeCells>
   <dataValidations count="5">

</xml_diff>

<commit_message>
Kich ban chi tiet: sua ten doi kem khu vuc/khoi thay vi chi tiet dia diem
</commit_message>
<xml_diff>
--- a/Quan_ly_hoi_thao_Final.xlsx
+++ b/Quan_ly_hoi_thao_Final.xlsx
@@ -10123,6 +10123,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1" s="31">
       <c r="A4" s="1" t="inlineStr">
         <is>
@@ -10235,10 +10236,10 @@
       <c r="C6" s="5" t="inlineStr">
         <is>
           <t>Vòng bảng Lượt 1, 4 trận song song:
-Sân 1 (Bảng A): Đội 10 (KV Yên Nghĩa/Văn Quán 2-3)  vs  Đội 4 (KV Đặng Thùy Trâm/Phạm Tuấn Tài 3/Láng Hạ/Mê Linh)
-Sân 2 (Bảng B): Đội 12 (KV Gia Lâm/Giải Phóng/Lê Thanh Nghị 2)  vs  Đội 1 (Trụ sở – Khối Sản xuất - Vận hành)
-Sân 3 (Bảng C): Đội 9 (KV Thanh Trì/Trần Đại Nghĩa 2/Lê Duẩn HP/Lạch Tray HP)  vs  Đội 3 (Trụ sở – Khối TNKH &amp; Truyền thông Marketing)
-Sân 4 (Bảng D): Đội 6 (KV Nguyễn Khuyến 1/Quang Trung/Văn Phú)  vs  Đội 7 (KV Văn Quán 1/Nguyễn Khuyến/Lê Thanh Nghị HD)</t>
+Sân 1 (Bảng A): Đội 10 (Khu vực HN10 - MB04 - MT02)  vs  Đội 4 (Khu vực HN01 - HN05 - MB05)
+Sân 2 (Bảng B): Đội 12 (Khu vực HN15)  vs  Đội 1 (Trụ sở – Khối Sản xuất - Vận hành)
+Sân 3 (Bảng C): Đội 9 (Khu vực HN07 - MB03)  vs  Đội 3 (Trụ sở – Khối Trải nghiệm khách hàng - hỗ trợ và truyền thông marketing)
+Sân 4 (Bảng D): Đội 6 (Khu vực HN02 - MB01)  vs  Đội 7 (Khu vực HN02 - MB01)</t>
         </is>
       </c>
       <c r="D6" s="10">
@@ -10283,10 +10284,10 @@
       <c r="C7" s="5" t="inlineStr">
         <is>
           <t>Vòng bảng Lượt 2, 4 trận song song:
-Sân 1 (Bảng A): Đội 10 (KV Yên Nghĩa/Văn Quán 2-3)  vs  Đội 5 (KV Trần Quốc Vượng/Xuân Thủy/Hoàng Quốc Việt/Bắc Từ Liêm)
-Sân 2 (Bảng B): Đội 12 (KV Gia Lâm/Giải Phóng/Lê Thanh Nghị 2)  vs  Đội 2 (Trụ sở – Khối Quản trị)
-Sân 3 (Bảng C): Đội 9 (KV Thanh Trì/Trần Đại Nghĩa 2/Lê Duẩn HP/Lạch Tray HP)  vs  Đội 8 (KV Thái Hà/Xuân Quỳnh/Tam Khương...)
-Sân 4 (Bảng D): Đội 6 (KV Nguyễn Khuyến 1/Quang Trung/Văn Phú)  vs  Đội 11 (KV Phùng Khoang/Bắc Sơn/MonBay/Hoàng Diệu/Phong Châu)</t>
+Sân 1 (Bảng A): Đội 10 (Khu vực HN10 - MB04 - MT02)  vs  Đội 5 (Khu vực HN06 - HN08)
+Sân 2 (Bảng B): Đội 12 (Khu vực HN15)  vs  Đội 2 (Trụ sở – Khối Quản trị)
+Sân 3 (Bảng C): Đội 9 (Khu vực HN07 - MB03)  vs  Đội 8 (Khu vực HN03 - HN11 - MB02 - MT01)
+Sân 4 (Bảng D): Đội 6 (Khu vực HN02 - MB01)  vs  Đội 11 (Khu vực HN10 - MB04 - MT02)</t>
         </is>
       </c>
       <c r="D7" s="10">
@@ -10331,10 +10332,10 @@
       <c r="C8" s="5" t="inlineStr">
         <is>
           <t>Vòng bảng Lượt 3, 4 trận song song:
-Sân 1 (Bảng A): Đội 4 (KV Đặng Thùy Trâm/Phạm Tuấn Tài 3/Láng Hạ/Mê Linh)  vs  Đội 5 (KV Trần Quốc Vượng/Xuân Thủy/Hoàng Quốc Việt/Bắc Từ Liêm)
+Sân 1 (Bảng A): Đội 4 (Khu vực HN01 - HN05 - MB05)  vs  Đội 5 (Khu vực HN06 - HN08)
 Sân 2 (Bảng B): Đội 1 (Trụ sở – Khối Sản xuất - Vận hành)  vs  Đội 2 (Trụ sở – Khối Quản trị)
-Sân 3 (Bảng C): Đội 3 (Trụ sở – Khối TNKH &amp; Truyền thông Marketing)  vs  Đội 8 (KV Thái Hà/Xuân Quỳnh/Tam Khương...)
-Sân 4 (Bảng D): Đội 7 (KV Văn Quán 1/Nguyễn Khuyến/Lê Thanh Nghị HD)  vs  Đội 11 (KV Phùng Khoang/Bắc Sơn/MonBay/Hoàng Diệu/Phong Châu)</t>
+Sân 3 (Bảng C): Đội 3 (Trụ sở – Khối Trải nghiệm khách hàng - hỗ trợ và truyền thông marketing)  vs  Đội 8 (Khu vực HN03 - HN11 - MB02 - MT01)
+Sân 4 (Bảng D): Đội 7 (Khu vực HN02 - MB01)  vs  Đội 11 (Khu vực HN10 - MB04 - MT02)</t>
         </is>
       </c>
       <c r="D8" s="10">
@@ -15416,17 +15417,17 @@
   <mergeCells count="14">
     <mergeCell ref="A169:G169"/>
     <mergeCell ref="A49:F49"/>
+    <mergeCell ref="A139:F139"/>
     <mergeCell ref="A94:F94"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A79:F79"/>
-    <mergeCell ref="A64:F64"/>
     <mergeCell ref="A34:F34"/>
     <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A139:F139"/>
+    <mergeCell ref="A124:F124"/>
     <mergeCell ref="A154:F154"/>
     <mergeCell ref="A19:G19"/>
     <mergeCell ref="A109:F109"/>
-    <mergeCell ref="A124:F124"/>
+    <mergeCell ref="A64:F64"/>
     <mergeCell ref="A17:H17"/>
   </mergeCells>
   <dataValidations count="5">

</xml_diff>